<commit_message>
Separa regime de caixa e competência e escapa texto do export
O fluxo de caixa somava transações pendentes/atrasadas como se o dinheiro
já tivesse entrado, e o DRE se dizia "regime de caixa" somando tudo.
Agora o fluxo de caixa usa só status Pago e o DRE é por competência,
cada um com o rótulo certo (Excel e HTML).

Também escapa descrição/categoria/status inseridos via innerHTML e o
"<" do JSON embutido, corrige comentários enganosos e atualiza README e
screenshots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SNGhJTcjeFguq5sm6ngrpK
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_financeiro.xlsx
+++ b/dashboard/dashboard_financeiro.xlsx
@@ -1326,21 +1326,21 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>TOTAL DE ENTRADAS</t>
+          <t>RECEBIDO (CAIXA)</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>TOTAL DE SAÍDAS</t>
+          <t>PAGO (CAIXA)</t>
         </is>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>SALDO DO PERÍODO</t>
+          <t>SALDO DE CAIXA</t>
         </is>
       </c>
       <c r="H4" s="5" t="n"/>
@@ -7133,7 +7133,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Período: Mar/2026 a Sep/2026 · valores somados a partir da aba Dados</t>
+          <t>Período: Mar/2026 a Sep/2026 · regime de caixa: só transações com status Pago (pendentes/atrasadas ficam em Contas a Pagar e Receber)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -7173,11 +7173,11 @@
         <v>46082</v>
       </c>
       <c r="B5" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
         <v/>
       </c>
       <c r="C5" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
         <v/>
       </c>
       <c r="D5" s="16">
@@ -7194,11 +7194,11 @@
         <v>46113</v>
       </c>
       <c r="B6" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
         <v/>
       </c>
       <c r="C6" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
         <v/>
       </c>
       <c r="D6" s="16">
@@ -7215,11 +7215,11 @@
         <v>46143</v>
       </c>
       <c r="B7" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
         <v/>
       </c>
       <c r="C7" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
         <v/>
       </c>
       <c r="D7" s="16">
@@ -7236,11 +7236,11 @@
         <v>46174</v>
       </c>
       <c r="B8" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
         <v/>
       </c>
       <c r="C8" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
         <v/>
       </c>
       <c r="D8" s="16">
@@ -7257,11 +7257,11 @@
         <v>46204</v>
       </c>
       <c r="B9" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
         <v/>
       </c>
       <c r="C9" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
         <v/>
       </c>
       <c r="D9" s="16">
@@ -7278,11 +7278,11 @@
         <v>46235</v>
       </c>
       <c r="B10" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
         <v/>
       </c>
       <c r="C10" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
         <v/>
       </c>
       <c r="D10" s="16">
@@ -7299,11 +7299,11 @@
         <v>46266</v>
       </c>
       <c r="B11" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
+        <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
         <v/>
       </c>
       <c r="D11" s="16">
@@ -10590,7 +10590,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Demonstrativo de Resultado — regime de caixa, a partir da aba Dados</t>
+          <t>Demonstrativo de Resultado — regime de competência (todas as transações lançadas, pagas ou não)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Prepara a planilha pra impressão e marca eixos dos gráficos como visíveis
Renderizando o Excel como ele sai impresso, as abas eram cortadas entre
páginas; agora cada uma cabe na largura de uma folha A4 deitada e a aba
Dados repete o cabeçalho. Os eixos dos 4 gráficos passam a ser marcados
como visíveis (o openpyxl 3.1 não grava essa marcação).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SNGhJTcjeFguq5sm6ngrpK
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_financeiro.xlsx
+++ b/dashboard/dashboard_financeiro.xlsx
@@ -13,7 +13,9 @@
     <sheet name="Contas a Pagar e Receber" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DRE" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dados'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -469,6 +471,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -480,6 +483,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -597,6 +601,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -608,6 +613,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -712,6 +718,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -723,6 +730,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -805,6 +813,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -816,6 +825,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -1277,7 +1287,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1442,6 +1452,7 @@
     <mergeCell ref="G7:I7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -1450,7 +1461,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7097,6 +7108,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -7107,7 +7119,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7349,6 +7361,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -7357,7 +7370,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -10556,6 +10569,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="2">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
@@ -10567,7 +10581,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -10729,6 +10743,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Grava o resultado das fórmulas e os dados dos gráficos na planilha
A planilha abria vazia em visualizadores que não calculam fórmulas
(celular, prévias online): o openpyxl grava a fórmula mas não o
resultado, e os gráficos sem a cópia dos dados. Cada fórmula agora leva
o resultado calculado em Python com a mesma regra (conferido contra o
LibreOffice recalculando do zero: 54 de 54 iguais) e cada gráfico leva
seus dados. A geração falha se alguma fórmula ficar sem resultado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SNGhJTcjeFguq5sm6ngrpK
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_financeiro.xlsx
+++ b/dashboard/dashboard_financeiro.xlsx
@@ -414,6 +414,12 @@
           <tx>
             <strRef>
               <f>'Fluxo Mensal'!B4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Entradas</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -427,11 +433,61 @@
           <cat>
             <numRef>
               <f>'Fluxo Mensal'!$A$5:$A$11</f>
+              <numCache>
+                <formatCode>mmm/yyyy</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>46082</v>
+                </pt>
+                <pt idx="1">
+                  <v>46113</v>
+                </pt>
+                <pt idx="2">
+                  <v>46143</v>
+                </pt>
+                <pt idx="3">
+                  <v>46174</v>
+                </pt>
+                <pt idx="4">
+                  <v>46204</v>
+                </pt>
+                <pt idx="5">
+                  <v>46235</v>
+                </pt>
+                <pt idx="6">
+                  <v>46266</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Fluxo Mensal'!$B$5:$B$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>0</v>
+                </pt>
+                <pt idx="1">
+                  <v>17510.88</v>
+                </pt>
+                <pt idx="2">
+                  <v>13227.69</v>
+                </pt>
+                <pt idx="3">
+                  <v>10106.95</v>
+                </pt>
+                <pt idx="4">
+                  <v>15254.72</v>
+                </pt>
+                <pt idx="5">
+                  <v>14949.33</v>
+                </pt>
+                <pt idx="6">
+                  <v>11926.98</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -441,6 +497,12 @@
           <tx>
             <strRef>
               <f>'Fluxo Mensal'!C4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Saídas</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -454,11 +516,61 @@
           <cat>
             <numRef>
               <f>'Fluxo Mensal'!$A$5:$A$11</f>
+              <numCache>
+                <formatCode>mmm/yyyy</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>46082</v>
+                </pt>
+                <pt idx="1">
+                  <v>46113</v>
+                </pt>
+                <pt idx="2">
+                  <v>46143</v>
+                </pt>
+                <pt idx="3">
+                  <v>46174</v>
+                </pt>
+                <pt idx="4">
+                  <v>46204</v>
+                </pt>
+                <pt idx="5">
+                  <v>46235</v>
+                </pt>
+                <pt idx="6">
+                  <v>46266</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Fluxo Mensal'!$C$5:$C$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>0</v>
+                </pt>
+                <pt idx="1">
+                  <v>3978.99</v>
+                </pt>
+                <pt idx="2">
+                  <v>9067.969999999999</v>
+                </pt>
+                <pt idx="3">
+                  <v>0</v>
+                </pt>
+                <pt idx="4">
+                  <v>24986.93</v>
+                </pt>
+                <pt idx="5">
+                  <v>6810.780000000001</v>
+                </pt>
+                <pt idx="6">
+                  <v>16794.63</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -544,6 +656,12 @@
           <tx>
             <strRef>
               <f>'Fluxo Mensal'!B4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Entradas</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -557,11 +675,61 @@
           <cat>
             <numRef>
               <f>'Fluxo Mensal'!$A$5:$A$11</f>
+              <numCache>
+                <formatCode>mmm/yyyy</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>46082</v>
+                </pt>
+                <pt idx="1">
+                  <v>46113</v>
+                </pt>
+                <pt idx="2">
+                  <v>46143</v>
+                </pt>
+                <pt idx="3">
+                  <v>46174</v>
+                </pt>
+                <pt idx="4">
+                  <v>46204</v>
+                </pt>
+                <pt idx="5">
+                  <v>46235</v>
+                </pt>
+                <pt idx="6">
+                  <v>46266</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Fluxo Mensal'!$B$5:$B$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>0</v>
+                </pt>
+                <pt idx="1">
+                  <v>17510.88</v>
+                </pt>
+                <pt idx="2">
+                  <v>13227.69</v>
+                </pt>
+                <pt idx="3">
+                  <v>10106.95</v>
+                </pt>
+                <pt idx="4">
+                  <v>15254.72</v>
+                </pt>
+                <pt idx="5">
+                  <v>14949.33</v>
+                </pt>
+                <pt idx="6">
+                  <v>11926.98</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -571,6 +739,12 @@
           <tx>
             <strRef>
               <f>'Fluxo Mensal'!C4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Saídas</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -584,11 +758,61 @@
           <cat>
             <numRef>
               <f>'Fluxo Mensal'!$A$5:$A$11</f>
+              <numCache>
+                <formatCode>mmm/yyyy</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>46082</v>
+                </pt>
+                <pt idx="1">
+                  <v>46113</v>
+                </pt>
+                <pt idx="2">
+                  <v>46143</v>
+                </pt>
+                <pt idx="3">
+                  <v>46174</v>
+                </pt>
+                <pt idx="4">
+                  <v>46204</v>
+                </pt>
+                <pt idx="5">
+                  <v>46235</v>
+                </pt>
+                <pt idx="6">
+                  <v>46266</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Fluxo Mensal'!$C$5:$C$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>0</v>
+                </pt>
+                <pt idx="1">
+                  <v>3978.99</v>
+                </pt>
+                <pt idx="2">
+                  <v>9067.969999999999</v>
+                </pt>
+                <pt idx="3">
+                  <v>0</v>
+                </pt>
+                <pt idx="4">
+                  <v>24986.93</v>
+                </pt>
+                <pt idx="5">
+                  <v>6810.780000000001</v>
+                </pt>
+                <pt idx="6">
+                  <v>16794.63</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -673,6 +897,12 @@
           <tx>
             <strRef>
               <f>'Fluxo Mensal'!E4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Saldo Acumulado</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -701,11 +931,61 @@
           <cat>
             <numRef>
               <f>'Fluxo Mensal'!$A$5:$A$11</f>
+              <numCache>
+                <formatCode>mmm/yyyy</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>46082</v>
+                </pt>
+                <pt idx="1">
+                  <v>46113</v>
+                </pt>
+                <pt idx="2">
+                  <v>46143</v>
+                </pt>
+                <pt idx="3">
+                  <v>46174</v>
+                </pt>
+                <pt idx="4">
+                  <v>46204</v>
+                </pt>
+                <pt idx="5">
+                  <v>46235</v>
+                </pt>
+                <pt idx="6">
+                  <v>46266</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Fluxo Mensal'!$E$5:$E$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="7"/>
+                <pt idx="0">
+                  <v>0</v>
+                </pt>
+                <pt idx="1">
+                  <v>13531.89</v>
+                </pt>
+                <pt idx="2">
+                  <v>17691.61</v>
+                </pt>
+                <pt idx="3">
+                  <v>27798.56</v>
+                </pt>
+                <pt idx="4">
+                  <v>18066.35</v>
+                </pt>
+                <pt idx="5">
+                  <v>26204.9</v>
+                </pt>
+                <pt idx="6">
+                  <v>21337.25</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -794,13 +1074,56 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'DRE'!$A$6:$A$11</f>
-            </numRef>
+              <strCache>
+                <ptCount val="6"/>
+                <pt idx="0">
+                  <v>Aluguel</v>
+                </pt>
+                <pt idx="1">
+                  <v>Fornecedor</v>
+                </pt>
+                <pt idx="2">
+                  <v>Imposto</v>
+                </pt>
+                <pt idx="3">
+                  <v>Manutenção</v>
+                </pt>
+                <pt idx="4">
+                  <v>Marketing</v>
+                </pt>
+                <pt idx="5">
+                  <v>Salário</v>
+                </pt>
+              </strCache>
+            </strRef>
           </cat>
           <val>
             <numRef>
               <f>'DRE'!$B$6:$B$11</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00</formatCode>
+                <ptCount val="6"/>
+                <pt idx="0">
+                  <v>26246.34</v>
+                </pt>
+                <pt idx="1">
+                  <v>46762.05</v>
+                </pt>
+                <pt idx="2">
+                  <v>68429.45</v>
+                </pt>
+                <pt idx="3">
+                  <v>28808.36</v>
+                </pt>
+                <pt idx="4">
+                  <v>25904.33</v>
+                </pt>
+                <pt idx="5">
+                  <v>47849.25</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -1359,19 +1682,19 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="7">
         <f>'Fluxo Mensal'!B12</f>
-        <v/>
+        <v>82976.55</v>
       </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="10">
         <f>'Fluxo Mensal'!C12</f>
-        <v/>
+        <v>61639.3</v>
       </c>
       <c r="E5" s="8" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="11">
         <f>'Fluxo Mensal'!D12</f>
-        <v/>
+        <v>21337.25</v>
       </c>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="9" t="n"/>
@@ -1402,19 +1725,19 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="7">
         <f>'Contas a Pagar e Receber'!D5</f>
-        <v/>
+        <v>199712.9</v>
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="10">
         <f>'Contas a Pagar e Receber'!D6</f>
-        <v/>
+        <v>177687.16</v>
       </c>
       <c r="E8" s="8" t="n"/>
       <c r="F8" s="9" t="n"/>
       <c r="G8" s="11">
         <f>DRE!B14</f>
-        <v/>
+        <v>61963.98</v>
       </c>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="9" t="n"/>
@@ -7186,19 +7509,19 @@
       </c>
       <c r="B5" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C5" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A5,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A5,1))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="D5" s="16">
         <f>B5-C5</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E5" s="16">
         <f>D5</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6">
@@ -7207,19 +7530,19 @@
       </c>
       <c r="B6" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
-        <v/>
+        <v>17510.88</v>
       </c>
       <c r="C6" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A6,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A6,1))</f>
-        <v/>
+        <v>3978.99</v>
       </c>
       <c r="D6" s="16">
         <f>B6-C6</f>
-        <v/>
+        <v>13531.89</v>
       </c>
       <c r="E6" s="16">
         <f>E5+D6</f>
-        <v/>
+        <v>13531.89</v>
       </c>
     </row>
     <row r="7">
@@ -7228,19 +7551,19 @@
       </c>
       <c r="B7" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
-        <v/>
+        <v>13227.69</v>
       </c>
       <c r="C7" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A7,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A7,1))</f>
-        <v/>
+        <v>9067.97</v>
       </c>
       <c r="D7" s="16">
         <f>B7-C7</f>
-        <v/>
+        <v>4159.72</v>
       </c>
       <c r="E7" s="16">
         <f>E6+D7</f>
-        <v/>
+        <v>17691.61</v>
       </c>
     </row>
     <row r="8">
@@ -7249,19 +7572,19 @@
       </c>
       <c r="B8" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
-        <v/>
+        <v>10106.95</v>
       </c>
       <c r="C8" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A8,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A8,1))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="D8" s="16">
         <f>B8-C8</f>
-        <v/>
+        <v>10106.95</v>
       </c>
       <c r="E8" s="16">
         <f>E7+D8</f>
-        <v/>
+        <v>27798.56</v>
       </c>
     </row>
     <row r="9">
@@ -7270,19 +7593,19 @@
       </c>
       <c r="B9" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
-        <v/>
+        <v>15254.72</v>
       </c>
       <c r="C9" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A9,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A9,1))</f>
-        <v/>
+        <v>24986.93</v>
       </c>
       <c r="D9" s="16">
         <f>B9-C9</f>
-        <v/>
+        <v>-9732.21</v>
       </c>
       <c r="E9" s="16">
         <f>E8+D9</f>
-        <v/>
+        <v>18066.35</v>
       </c>
     </row>
     <row r="10">
@@ -7291,19 +7614,19 @@
       </c>
       <c r="B10" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
-        <v/>
+        <v>14949.33</v>
       </c>
       <c r="C10" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A10,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A10,1))</f>
-        <v/>
+        <v>6810.78</v>
       </c>
       <c r="D10" s="16">
         <f>B10-C10</f>
-        <v/>
+        <v>8138.55</v>
       </c>
       <c r="E10" s="16">
         <f>E9+D10</f>
-        <v/>
+        <v>26204.9</v>
       </c>
     </row>
     <row r="11">
@@ -7312,19 +7635,19 @@
       </c>
       <c r="B11" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
-        <v/>
+        <v>11926.98</v>
       </c>
       <c r="C11" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pago",Dados!$A$2:$A$201,"&gt;="&amp;A11,Dados!$A$2:$A$201,"&lt;"&amp;EDATE(A11,1))</f>
-        <v/>
+        <v>16794.63</v>
       </c>
       <c r="D11" s="16">
         <f>B11-C11</f>
-        <v/>
+        <v>-4867.65</v>
       </c>
       <c r="E11" s="16">
         <f>E10+D11</f>
-        <v/>
+        <v>21337.25</v>
       </c>
     </row>
     <row r="12">
@@ -7335,15 +7658,15 @@
       </c>
       <c r="B12" s="19">
         <f>SUM(B5:B11)</f>
-        <v/>
+        <v>82976.55</v>
       </c>
       <c r="C12" s="19">
         <f>SUM(C5:C11)</f>
-        <v/>
+        <v>61639.3</v>
       </c>
       <c r="D12" s="19">
         <f>SUM(D5:D11)</f>
-        <v/>
+        <v>21337.25</v>
       </c>
       <c r="E12" s="20" t="n"/>
     </row>
@@ -7446,15 +7769,15 @@
       </c>
       <c r="B5" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Pendente")</f>
-        <v/>
+        <v>86550.82</v>
       </c>
       <c r="C5" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada",Dados!$F$2:$F$201,"Atrasado")</f>
-        <v/>
+        <v>113162.08</v>
       </c>
       <c r="D5" s="25">
         <f>B5+C5</f>
-        <v/>
+        <v>199712.9</v>
       </c>
     </row>
     <row r="6">
@@ -7465,15 +7788,15 @@
       </c>
       <c r="B6" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Pendente")</f>
-        <v/>
+        <v>84201.8</v>
       </c>
       <c r="C6" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$F$2:$F$201,"Atrasado")</f>
-        <v/>
+        <v>93485.36</v>
       </c>
       <c r="D6" s="25">
         <f>B6+C6</f>
-        <v/>
+        <v>177687.16</v>
       </c>
     </row>
     <row r="7">
@@ -7486,7 +7809,7 @@
       <c r="C7" s="27" t="n"/>
       <c r="D7" s="28">
         <f>D5-D6</f>
-        <v/>
+        <v>22025.74</v>
       </c>
     </row>
     <row r="10">
@@ -10620,7 +10943,7 @@
       </c>
       <c r="B4" s="33">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Entrada")</f>
-        <v/>
+        <v>305963.76</v>
       </c>
     </row>
     <row r="5">
@@ -10638,7 +10961,7 @@
       </c>
       <c r="B6" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Aluguel")</f>
-        <v/>
+        <v>26246.34</v>
       </c>
     </row>
     <row r="7">
@@ -10649,7 +10972,7 @@
       </c>
       <c r="B7" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Fornecedor")</f>
-        <v/>
+        <v>46762.05</v>
       </c>
     </row>
     <row r="8">
@@ -10660,7 +10983,7 @@
       </c>
       <c r="B8" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Imposto")</f>
-        <v/>
+        <v>68429.45</v>
       </c>
     </row>
     <row r="9">
@@ -10671,7 +10994,7 @@
       </c>
       <c r="B9" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Manutenção")</f>
-        <v/>
+        <v>28808.36</v>
       </c>
     </row>
     <row r="10">
@@ -10682,7 +11005,7 @@
       </c>
       <c r="B10" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Marketing")</f>
-        <v/>
+        <v>25904.33</v>
       </c>
     </row>
     <row r="11">
@@ -10693,7 +11016,7 @@
       </c>
       <c r="B11" s="16">
         <f>SUMIFS(Dados!$E$2:$E$201,Dados!$D$2:$D$201,"Saída",Dados!$C$2:$C$201,"Salário")</f>
-        <v/>
+        <v>47849.25</v>
       </c>
     </row>
     <row r="12">
@@ -10704,7 +11027,7 @@
       </c>
       <c r="B12" s="35">
         <f>SUM(B6:B11)</f>
-        <v/>
+        <v>243999.78</v>
       </c>
     </row>
     <row r="14">
@@ -10715,7 +11038,7 @@
       </c>
       <c r="B14" s="37">
         <f>B4-B12</f>
-        <v/>
+        <v>61963.98</v>
       </c>
     </row>
     <row r="15">
@@ -10726,7 +11049,7 @@
       </c>
       <c r="B15" s="39">
         <f>B14/B4</f>
-        <v/>
+        <v>0.2025206515</v>
       </c>
     </row>
   </sheetData>

</xml_diff>